<commit_message>
Reframe target users as students studying on campus with 15-minute breaks between periods; drop dormitory premise
</commit_message>
<xml_diff>
--- a/02-P1-nghien-cuu/khao-sat/ket-qua-khao-sat-MO-PHONG.xlsx
+++ b/02-P1-nghien-cuu/khao-sat/ket-qua-khao-sat-MO-PHONG.xlsx
@@ -67,13 +67,13 @@
     <t>Q2 Nơi ở</t>
   </si>
   <si>
-    <t>Q3 Số slot/ngày</t>
+    <t>Q3 Số tiết/ngày</t>
   </si>
   <si>
     <t>Q4 Điện thoại</t>
   </si>
   <si>
-    <t>Q5 Phút nghỉ giữa 2 slot</t>
+    <t>Q5 Phút nghỉ giữa 2 tiết</t>
   </si>
   <si>
     <t>Q6 Di chuyển giữa phòng</t>

</xml_diff>

<commit_message>
Keep 'slot' wording for class periods; only the dormitory premise stays removed
</commit_message>
<xml_diff>
--- a/02-P1-nghien-cuu/khao-sat/ket-qua-khao-sat-MO-PHONG.xlsx
+++ b/02-P1-nghien-cuu/khao-sat/ket-qua-khao-sat-MO-PHONG.xlsx
@@ -67,13 +67,13 @@
     <t>Q2 Nơi ở</t>
   </si>
   <si>
-    <t>Q3 Số tiết/ngày</t>
+    <t>Q3 Số slot/ngày</t>
   </si>
   <si>
     <t>Q4 Điện thoại</t>
   </si>
   <si>
-    <t>Q5 Phút nghỉ giữa 2 tiết</t>
+    <t>Q5 Phút nghỉ giữa 2 slot</t>
   </si>
   <si>
     <t>Q6 Di chuyển giữa phòng</t>

</xml_diff>